<commit_message>
Delete record: メドレー 200m
</commit_message>
<xml_diff>
--- a/穂果記録.xlsx
+++ b/穂果記録.xlsx
@@ -1804,7 +1804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1997,35 +1997,9 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>125.01</v>
+        <v>171.01</v>
       </c>
       <c r="F7" t="inlineStr">
-        <is>
-          <t>荒野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>小6</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>200</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>171.01</v>
-      </c>
-      <c r="F8" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>

</xml_diff>

<commit_message>
Add record: ブレ 100m
</commit_message>
<xml_diff>
--- a/穂果記録.xlsx
+++ b/穂果記録.xlsx
@@ -8,9 +8,9 @@
   <sheets>
     <sheet name="バッタ" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="バック" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ブレ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="メドレー" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="フリー" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="メドレー" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="フリー" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ブレ" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1042,369 +1042,183 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.8984375" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="15.796875" bestFit="1" customWidth="1" style="9" min="1" max="1"/>
-    <col width="14.8984375" customWidth="1" style="1" min="2" max="10"/>
-    <col width="9.8984375" customWidth="1" style="1" min="11" max="11"/>
-    <col width="14.8984375" customWidth="1" style="1" min="12" max="16384"/>
-  </cols>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>日付</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>学年</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>距離</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>長水路 or 短水路</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>長水路or短水路</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>タイム</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>会場</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
-        <v>45788</v>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>58.87</v>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
+      <c r="A2" s="11" t="n">
+        <v>45710</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>小4</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>200</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4'43"09</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
-        <v>45815</v>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>55.01</v>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
+      <c r="A3" s="11" t="n">
+        <v>45808</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>200</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4'02"71</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>45844</v>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>52.08</v>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
+      <c r="A4" s="11" t="n">
+        <v>45899</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>200</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3'37"53</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>45942</v>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>52.97</v>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="J5" s="1" t="inlineStr">
+      <c r="A5" s="11" t="n">
+        <v>45991</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>200</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3'21"34</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>45955</v>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>49.74</v>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>45984</v>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>49.06</v>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>45984</v>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>1'41"11</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>46033</v>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="n">
-        <v>47.55</v>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
-        <v>46053</v>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="n">
-        <v>46.9</v>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="n">
-        <v>47.42</v>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>小6</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="n">
-        <v>47.95</v>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="A6" s="11" t="n">
+        <v>46081</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>200</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3'14"47</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="G2:G5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$I$5:$I$6</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F12" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$J$5:$J$6</formula1>
-    </dataValidation>
-    <dataValidation sqref="D2:D180" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$J$2:$J$3</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1414,7 +1228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1451,35 +1265,33 @@
     </row>
     <row r="2">
       <c r="A2" s="11" t="n">
-        <v>45710</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4'43"09</t>
-        </is>
+      <c r="E2" t="n">
+        <v>47.91</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="n">
-        <v>45808</v>
+        <v>45816</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1487,27 +1299,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>4'02"71</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>47.54</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
-        <v>45899</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1515,27 +1325,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>3'37"53</t>
-        </is>
+      <c r="E4" t="n">
+        <v>44.48</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>45991</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1543,27 +1351,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>3'21"34</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>44.39</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
-        <v>46081</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1571,19 +1377,147 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>3'14"47</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>40.39</v>
       </c>
       <c r="F6" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="n">
+        <v>45955</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>39.07</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="n">
+        <v>46053</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>38.24</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="n">
+        <v>46074</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>37.73</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小6</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>40.28</v>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>
@@ -1600,7 +1534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1653,7 +1587,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>47.91</v>
+        <v>58.87</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1663,7 +1597,7 @@
     </row>
     <row r="3">
       <c r="A3" s="11" t="n">
-        <v>45816</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1679,7 +1613,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>47.54</v>
+        <v>55.01</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1689,7 +1623,7 @@
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
-        <v>45823</v>
+        <v>45844</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1701,11 +1635,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>44.48</v>
+        <v>52.08</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1715,7 +1649,7 @@
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>45844</v>
+        <v>45942</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1731,7 +1665,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>44.39</v>
+        <v>52.97</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1741,7 +1675,7 @@
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
-        <v>45942</v>
+        <v>45955</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1753,11 +1687,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>40.39</v>
+        <v>49.74</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1767,7 +1701,7 @@
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">
-        <v>45955</v>
+        <v>45984</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1779,11 +1713,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>40.5</v>
+        <v>49.06</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1793,7 +1727,7 @@
     </row>
     <row r="8">
       <c r="A8" s="11" t="n">
-        <v>46033</v>
+        <v>45984</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1801,15 +1735,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>39.07</v>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1'41"11</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1819,7 +1755,7 @@
     </row>
     <row r="9">
       <c r="A9" s="11" t="n">
-        <v>46053</v>
+        <v>46033</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1835,7 +1771,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>38.24</v>
+        <v>47.55</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1845,7 +1781,7 @@
     </row>
     <row r="10">
       <c r="A10" s="11" t="n">
-        <v>46074</v>
+        <v>46053</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1857,11 +1793,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>37.73</v>
+        <v>46.9</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1871,27 +1807,79 @@
     </row>
     <row r="11">
       <c r="A11" s="11" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>47.42</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n">
         <v>46130</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>小6</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>40.28</v>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>47.95</v>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n">
+        <v>46053</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>100</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>99.48999999999999</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Delete record: ブレ 100m
</commit_message>
<xml_diff>
--- a/穂果記録.xlsx
+++ b/穂果記録.xlsx
@@ -1534,7 +1534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1883,32 +1883,6 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="11" t="n">
-        <v>46053</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>100</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>99.48999999999999</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add record: メドレー 50m
</commit_message>
<xml_diff>
--- a/穂果記録.xlsx
+++ b/穂果記録.xlsx
@@ -8,9 +8,9 @@
   <sheets>
     <sheet name="バッタ" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="バック" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="メドレー" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ブレ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="フリー" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ブレ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="フリー" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="メドレー" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1042,7 +1042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1079,35 +1079,33 @@
     </row>
     <row r="2">
       <c r="A2" s="11" t="n">
-        <v>45710</v>
+        <v>45788</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小4</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4'43"09</t>
-        </is>
+      <c r="E2" t="n">
+        <v>58.87</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="n">
-        <v>45808</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1115,27 +1113,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>4'02"71</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>55.01</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
-        <v>45899</v>
+        <v>45844</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1143,27 +1139,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>3'37"53</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>52.08</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>45991</v>
+        <v>45942</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1171,27 +1165,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>3'21"34</t>
-        </is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>52.97</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
-        <v>46081</v>
+        <v>45955</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1199,21 +1191,203 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>3'14"47</t>
-        </is>
+      <c r="E6" t="n">
+        <v>49.74</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="n">
+        <v>45984</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>49.06</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="n">
+        <v>45984</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>100</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1'41"11</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>47.55</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="n">
+        <v>46053</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>47.42</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>小6</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>47.95</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n">
+        <v>46053</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>100</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>99.48999999999999</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1281,7 +1455,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>58.87</v>
+        <v>47.91</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1291,7 +1465,7 @@
     </row>
     <row r="3">
       <c r="A3" s="11" t="n">
-        <v>45815</v>
+        <v>45816</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1307,7 +1481,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>55.01</v>
+        <v>47.54</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1317,7 +1491,7 @@
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
-        <v>45844</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1329,11 +1503,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52.08</v>
+        <v>44.48</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1343,7 +1517,7 @@
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>45942</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1359,7 +1533,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>52.97</v>
+        <v>44.39</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1369,7 +1543,7 @@
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
-        <v>45955</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1381,11 +1555,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>49.74</v>
+        <v>40.39</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1395,7 +1569,7 @@
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">
-        <v>45984</v>
+        <v>45955</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1407,11 +1581,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>49.06</v>
+        <v>40.5</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1421,7 +1595,7 @@
     </row>
     <row r="8">
       <c r="A8" s="11" t="n">
-        <v>45984</v>
+        <v>46033</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1429,17 +1603,15 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>1'41"11</t>
-        </is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>39.07</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1449,7 +1621,7 @@
     </row>
     <row r="9">
       <c r="A9" s="11" t="n">
-        <v>46033</v>
+        <v>46053</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1465,7 +1637,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>47.55</v>
+        <v>38.24</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1475,7 +1647,7 @@
     </row>
     <row r="10">
       <c r="A10" s="11" t="n">
-        <v>46053</v>
+        <v>46074</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1487,11 +1659,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>46.9</v>
+        <v>37.73</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1501,11 +1673,11 @@
     </row>
     <row r="11">
       <c r="A11" s="11" t="n">
-        <v>46075</v>
+        <v>46130</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小6</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1513,67 +1685,15 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>47.42</v>
+        <v>40.28</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>小6</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>47.95</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
           <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="n">
-        <v>46053</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>100</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>99.48999999999999</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1625,33 +1745,35 @@
     </row>
     <row r="2">
       <c r="A2" s="11" t="n">
-        <v>45788</v>
+        <v>45710</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小4</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>47.91</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4'43"09</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="n">
-        <v>45816</v>
+        <v>45808</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1659,25 +1781,27 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>47.54</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4'02"71</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
-        <v>45823</v>
+        <v>45899</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1685,25 +1809,27 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>短水路</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>44.48</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3'37"53</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>45844</v>
+        <v>45991</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1711,25 +1837,27 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>44.39</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3'21"34</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
-        <v>45942</v>
+        <v>46081</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1737,29 +1865,31 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>40.39</v>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3'14"47</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">
-        <v>45955</v>
+        <v>46145</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小6</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1771,113 +1901,9 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>40.5</v>
+        <v>173.24</v>
       </c>
       <c r="F7" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="n">
-        <v>46033</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>50</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>39.07</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="n">
-        <v>46053</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>50</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>38.24</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="n">
-        <v>46074</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>37.73</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="n">
-        <v>46130</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>小6</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>40.28</v>
-      </c>
-      <c r="F11" t="inlineStr">
         <is>
           <t>菰野スイミング</t>
         </is>

</xml_diff>

<commit_message>
Edit record: ブレ 50m
</commit_message>
<xml_diff>
--- a/穂果記録.xlsx
+++ b/穂果記録.xlsx
@@ -9,8 +9,8 @@
     <sheet name="バッタ" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="バック" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="メドレー" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ブレ" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="フリー" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="フリー" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ブレ" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1254,7 +1254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>58.87</v>
+        <v>47.91</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1317,7 +1317,7 @@
     </row>
     <row r="3">
       <c r="A3" s="11" t="n">
-        <v>45815</v>
+        <v>45816</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>55.01</v>
+        <v>47.54</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1343,7 +1343,7 @@
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
-        <v>45844</v>
+        <v>45823</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1355,11 +1355,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>52.08</v>
+        <v>44.48</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1369,7 +1369,7 @@
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>45942</v>
+        <v>45844</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>52.97</v>
+        <v>44.39</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1395,7 +1395,7 @@
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
-        <v>45955</v>
+        <v>45942</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1407,11 +1407,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>49.74</v>
+        <v>40.39</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">
-        <v>45984</v>
+        <v>45955</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1433,11 +1433,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>49.06</v>
+        <v>40.5</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1447,7 +1447,7 @@
     </row>
     <row r="8">
       <c r="A8" s="11" t="n">
-        <v>45984</v>
+        <v>46033</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1455,17 +1455,15 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>長水路</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>1'41"11</t>
-        </is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>39.07</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1475,7 +1473,7 @@
     </row>
     <row r="9">
       <c r="A9" s="11" t="n">
-        <v>46033</v>
+        <v>46053</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1491,7 +1489,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>47.55</v>
+        <v>38.24</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1501,7 +1499,7 @@
     </row>
     <row r="10">
       <c r="A10" s="11" t="n">
-        <v>46053</v>
+        <v>46074</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1513,11 +1511,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>46.9</v>
+        <v>37.73</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1527,11 +1525,11 @@
     </row>
     <row r="11">
       <c r="A11" s="11" t="n">
-        <v>46075</v>
+        <v>46130</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>小5</t>
+          <t>小6</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1539,21 +1537,21 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>47.42</v>
+        <v>40.28</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>鈴鹿</t>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n">
-        <v>46130</v>
+        <v>46152</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1569,63 +1567,11 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>47.95</v>
+        <v>36.55</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="n">
-        <v>46053</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>小5</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>100</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>99.48999999999999</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="n">
-        <v>46152</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>小6</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>50</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>45.36</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1693,7 +1639,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>47.91</v>
+        <v>58.87</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1703,7 +1649,7 @@
     </row>
     <row r="3">
       <c r="A3" s="11" t="n">
-        <v>45816</v>
+        <v>45815</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -1719,7 +1665,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>47.54</v>
+        <v>55.01</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1729,7 +1675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="11" t="n">
-        <v>45823</v>
+        <v>45844</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -1741,11 +1687,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>44.48</v>
+        <v>52.08</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1755,7 +1701,7 @@
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>45844</v>
+        <v>45942</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -1771,7 +1717,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>44.39</v>
+        <v>52.97</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1781,7 +1727,7 @@
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
-        <v>45942</v>
+        <v>45955</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1793,11 +1739,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>40.39</v>
+        <v>49.74</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1807,7 +1753,7 @@
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">
-        <v>45955</v>
+        <v>45984</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1819,11 +1765,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>40.5</v>
+        <v>49.06</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1833,7 +1779,7 @@
     </row>
     <row r="8">
       <c r="A8" s="11" t="n">
-        <v>46033</v>
+        <v>45984</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1841,15 +1787,17 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>39.07</v>
+          <t>長水路</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1'41"11</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1859,7 +1807,7 @@
     </row>
     <row r="9">
       <c r="A9" s="11" t="n">
-        <v>46053</v>
+        <v>46033</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1875,7 +1823,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>38.24</v>
+        <v>47.55</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1885,7 +1833,7 @@
     </row>
     <row r="10">
       <c r="A10" s="11" t="n">
-        <v>46074</v>
+        <v>46053</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1897,11 +1845,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>長水路</t>
+          <t>短水路</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>37.73</v>
+        <v>46.9</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1911,11 +1859,11 @@
     </row>
     <row r="11">
       <c r="A11" s="11" t="n">
-        <v>46130</v>
+        <v>46075</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>小6</t>
+          <t>小5</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1923,41 +1871,93 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>短水路</t>
+          <t>長水路</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>40.28</v>
+        <v>47.42</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>菰野スイミング</t>
+          <t>鈴鹿</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>小6</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>47.95</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n">
+        <v>46053</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>100</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>99.48999999999999</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>鈴鹿</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="n">
         <v>46152</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>小6</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>短水路</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>36.55</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>鈴鹿</t>
+      <c r="C14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>短水路</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>45.36</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>菰野スイミング</t>
         </is>
       </c>
     </row>

</xml_diff>